<commit_message>
PositionSignal v1.1.0: wave/segment comparisons, association ownership, POP/POD
Declared wave and segment comparisons with independent-sample intervals
and repeated-respondent warnings; association-leadership reporting;
points-of-parity/points-of-difference candidates with configurable
descriptive thresholds. 31 tests.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/ratings_template.xlsx
+++ b/examples/ratings_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ratings" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ratings'!$A$1:$K$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ratings'!$A$1:$M$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,20 +427,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -451,50 +453,60 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>collection_wave</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>segment</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>brand</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>quality</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>value_for_money</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>innovation</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>style</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>sustainability</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>comfort</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>performance</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>exclusivity</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>sample_weight</t>
         </is>
@@ -508,34 +520,44 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Brand A</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>6</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F2" t="n">
         <v>4</v>
       </c>
-      <c r="E2" t="n">
-        <v>6</v>
-      </c>
-      <c r="F2" t="n">
-        <v>5</v>
-      </c>
       <c r="G2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="n">
         <v>4</v>
       </c>
-      <c r="H2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I2" t="n">
-        <v>6</v>
-      </c>
       <c r="J2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M2" t="n">
         <v>0.9</v>
       </c>
     </row>
@@ -547,34 +569,44 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Brand B</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D3" t="n">
-        <v>6</v>
-      </c>
       <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" t="n">
         <v>4</v>
       </c>
-      <c r="F3" t="n">
-        <v>6</v>
-      </c>
-      <c r="G3" t="n">
-        <v>5</v>
-      </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I3" t="n">
         <v>5</v>
       </c>
       <c r="J3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L3" t="n">
         <v>4</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>0.9</v>
       </c>
     </row>
@@ -586,34 +618,44 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Wave 1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Brand C</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D4" t="n">
-        <v>5</v>
-      </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" t="n">
         <v>4</v>
       </c>
-      <c r="G4" t="n">
-        <v>6</v>
-      </c>
-      <c r="H4" t="n">
-        <v>6</v>
-      </c>
       <c r="I4" t="n">
         <v>6</v>
       </c>
       <c r="J4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M4" t="n">
         <v>0.9</v>
       </c>
     </row>
@@ -625,34 +667,44 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Wave 2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Brand A</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="E5" t="n">
         <v>7</v>
       </c>
-      <c r="D5" t="n">
+      <c r="F5" t="n">
         <v>4</v>
       </c>
-      <c r="E5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F5" t="n">
-        <v>5</v>
-      </c>
       <c r="G5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" t="n">
         <v>4</v>
       </c>
-      <c r="H5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K5" t="n">
         <v>7</v>
       </c>
-      <c r="J5" t="n">
-        <v>5</v>
-      </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
+        <v>5</v>
+      </c>
+      <c r="M5" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -664,27 +716,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Wave 2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Brand B</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" t="n">
-        <v>6</v>
-      </c>
       <c r="E6" t="n">
         <v>5</v>
       </c>
       <c r="F6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" t="n">
         <v>7</v>
       </c>
-      <c r="G6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H6" t="n">
-        <v>5</v>
-      </c>
       <c r="I6" t="n">
         <v>5</v>
       </c>
@@ -692,6 +748,12 @@
         <v>5</v>
       </c>
       <c r="K6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M6" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -703,27 +765,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>Wave 2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Brand C</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D7" t="n">
-        <v>5</v>
-      </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" t="n">
         <v>4</v>
       </c>
-      <c r="G7" t="n">
-        <v>6</v>
-      </c>
-      <c r="H7" t="n">
-        <v>6</v>
-      </c>
       <c r="I7" t="n">
         <v>6</v>
       </c>
@@ -731,11 +797,17 @@
         <v>6</v>
       </c>
       <c r="K7" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" t="n">
+        <v>6</v>
+      </c>
+      <c r="M7" t="n">
         <v>1.1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K7"/>
+  <autoFilter ref="A1:M7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>